<commit_message>
vixlens-catalogo 0.12.2: selo Montagem lente pronta R$15 volta, ligado no modelo com combo
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo_com_combo.xlsx
+++ b/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo_com_combo.xlsx
@@ -1209,7 +1209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1959,37 +1959,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -3262,7 +3231,7 @@
       </c>
       <c r="M17" s="21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="N17" s="21" t="inlineStr">
@@ -3333,7 +3302,7 @@
       </c>
       <c r="M18" s="21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="N18" s="21" t="inlineStr">

</xml_diff>

<commit_message>
promovix: residual verde no 0276 e no 0257 do combo (modelo com combo)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo_com_combo.xlsx
+++ b/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo_com_combo.xlsx
@@ -4608,7 +4608,11 @@
       <c r="D4" s="56" t="n">
         <v>49.9</v>
       </c>
-      <c r="E4" s="57" t="n"/>
+      <c r="E4" s="57" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
       <c r="F4" s="57" t="n"/>
     </row>
     <row r="5">
@@ -4630,7 +4634,11 @@
       <c r="D5" s="56" t="n">
         <v>129.9</v>
       </c>
-      <c r="E5" s="57" t="n"/>
+      <c r="E5" s="57" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
       <c r="F5" s="57" t="n"/>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
promovix: residual verde nos combos Kodak e Essilor (8349, 8350, 8365, 0424)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo_com_combo.xlsx
+++ b/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo_com_combo.xlsx
@@ -943,7 +943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="B2:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -951,7 +951,6 @@
     <col width="92" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -966,7 +965,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -1034,7 +1032,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -1090,7 +1087,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
@@ -1158,7 +1154,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="B25" s="3" t="inlineStr">
         <is>
@@ -4665,7 +4660,11 @@
       <c r="D6" s="56" t="n">
         <v>50</v>
       </c>
-      <c r="E6" s="57" t="n"/>
+      <c r="E6" s="57" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
       <c r="F6" s="57" t="inlineStr">
         <is>
           <t>Também está em LENTE PRONTA KODAK.</t>
@@ -4691,7 +4690,11 @@
       <c r="D7" s="56" t="n">
         <v>65</v>
       </c>
-      <c r="E7" s="57" t="n"/>
+      <c r="E7" s="57" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
       <c r="F7" s="57" t="inlineStr">
         <is>
           <t>Também está em LENTE PRONTA KODAK.</t>
@@ -4717,7 +4720,11 @@
       <c r="D8" s="56" t="n">
         <v>179</v>
       </c>
-      <c r="E8" s="57" t="n"/>
+      <c r="E8" s="57" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
       <c r="F8" s="57" t="inlineStr">
         <is>
           <t>Também está em LENTE PRONTA KODAK.</t>
@@ -4743,7 +4750,11 @@
       <c r="D9" s="56" t="n">
         <v>119.9</v>
       </c>
-      <c r="E9" s="57" t="n"/>
+      <c r="E9" s="57" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
       <c r="F9" s="57" t="inlineStr">
         <is>
           <t>Também está em LENTE PRONTA ESSILOR.</t>

</xml_diff>